<commit_message>
more drop bar mtb
</commit_message>
<xml_diff>
--- a/data/gravel/Chaparral Titanium Angeles 2026.xlsx
+++ b/data/gravel/Chaparral Titanium Angeles 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/walker/Documents/Github/Bike Geometry Project/data/gravel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CCA8E01-7FA0-7046-A486-66D6A7AA0FAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{390AADF1-0135-D143-A4BC-56A343CBD2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3040" yWindow="1360" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -134,9 +134,6 @@
     <t>material</t>
   </si>
   <si>
-    <t>carbon</t>
-  </si>
-  <si>
     <t>udh</t>
   </si>
   <si>
@@ -429,6 +426,9 @@
   </si>
   <si>
     <t>Claremont, California, USA</t>
+  </si>
+  <si>
+    <t>titanium</t>
   </si>
 </sst>
 </file>
@@ -786,7 +786,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -794,7 +794,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -818,12 +818,12 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -831,7 +831,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -839,16 +839,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" t="s">
         <v>87</v>
-      </c>
-      <c r="E8" t="s">
-        <v>88</v>
       </c>
       <c r="F8" t="s">
         <v>7</v>
@@ -859,7 +859,7 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C9">
         <v>636.45000000000005</v>
@@ -879,7 +879,7 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C10">
         <v>379.5</v>
@@ -899,7 +899,7 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C11">
         <v>430</v>
@@ -919,7 +919,7 @@
         <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C12">
         <v>568</v>
@@ -936,10 +936,10 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C13">
         <v>26.7</v>
@@ -959,7 +959,7 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C14">
         <v>70.5</v>
@@ -979,7 +979,7 @@
         <v>12</v>
       </c>
       <c r="B15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C15">
         <v>73.5</v>
@@ -999,7 +999,7 @@
         <v>10</v>
       </c>
       <c r="B16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C16">
         <v>110</v>
@@ -1019,7 +1019,7 @@
         <v>18</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C17">
         <v>70</v>
@@ -1036,10 +1036,10 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C18">
         <v>302</v>
@@ -1059,7 +1059,7 @@
         <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C19">
         <v>452</v>
@@ -1076,10 +1076,10 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B20" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C20">
         <v>446.6</v>
@@ -1096,10 +1096,10 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C21">
         <v>630.70000000000005</v>
@@ -1116,10 +1116,10 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B22" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C22">
         <v>626.79999999999995</v>
@@ -1139,7 +1139,7 @@
         <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C23">
         <v>1073.3</v>
@@ -1156,10 +1156,10 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B24" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C24">
         <v>85</v>
@@ -1176,10 +1176,10 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B25" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C25">
         <v>80.2</v>
@@ -1196,10 +1196,10 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B26" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C26">
         <v>26.8</v>
@@ -1219,7 +1219,7 @@
         <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C27">
         <v>44</v>
@@ -1239,7 +1239,7 @@
         <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C28">
         <v>493</v>
@@ -1256,7 +1256,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C29">
         <v>100</v>
@@ -1273,7 +1273,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C30">
         <v>20</v>
@@ -1388,26 +1388,26 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
@@ -1415,25 +1415,25 @@
         <v>32</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>33</v>
+        <v>127</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
+        <v>33</v>
+      </c>
+      <c r="B47" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B49">
         <v>2.4</v>
@@ -1441,12 +1441,12 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B51" s="1">
         <v>100</v>
@@ -1454,7 +1454,7 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B52">
         <v>100</v>
@@ -1462,17 +1462,17 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B55">
         <v>148</v>
@@ -1480,64 +1480,64 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B63" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B65">
         <v>30.9</v>
@@ -1545,15 +1545,15 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B67">
         <v>42</v>
@@ -1562,7 +1562,7 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B68">
         <v>50</v>
@@ -1570,82 +1570,82 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B72" s="1"/>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B75" s="1"/>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B83">
         <v>2500</v>
@@ -1653,28 +1653,28 @@
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>